<commit_message>
Working on housing 	- Remove screw nut for pressure compensation element 	- Add thread for presure compensation element 	- Change spacer 	- Change screws 	- Change the housing in the BOM to the light gray version 	- Finalize housing
Misc:
	- Print new BOM PDF
	- Add drawing for the housing

Signed-off-by: Daniel Kampert <DanielKampert@kampis-elektroecke.de>
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23001"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC30F405-3543-49CD-8F53-7A2B4281DF36}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10CF5FF0-DF75-4044-806F-DE9254F27BE5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stückliste" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="303">
   <si>
     <t>Nicht bestückt</t>
   </si>
@@ -688,18 +688,6 @@
   </si>
   <si>
     <t>Bopla</t>
-  </si>
-  <si>
-    <t>B 080805 PC-V0-G 7024</t>
-  </si>
-  <si>
-    <t>Distanzhülse</t>
-  </si>
-  <si>
-    <t>Harwin</t>
-  </si>
-  <si>
-    <t>R30-6701494</t>
   </si>
   <si>
     <t>Druckausgleichselemen</t>
@@ -1082,21 +1070,6 @@
     <t>TE</t>
   </si>
   <si>
-    <t>Schraube M3x18</t>
-  </si>
-  <si>
-    <t>Mutter M6x0.75</t>
-  </si>
-  <si>
-    <t>1-1634816-0</t>
-  </si>
-  <si>
-    <t>RS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1-1634816-0 </t>
-  </si>
-  <si>
     <t>R8</t>
   </si>
   <si>
@@ -1307,15 +1280,9 @@
     <t>3.556000</t>
   </si>
   <si>
-    <t>SHR-ZYL-ISO14580-A2/70-TX10-M3X18</t>
-  </si>
-  <si>
     <t>Würth</t>
   </si>
   <si>
-    <t>855-R30-6701494</t>
-  </si>
-  <si>
     <t>4-in-1 sensor, gas, humidity, pressure, temperature</t>
   </si>
   <si>
@@ -1509,6 +1476,30 @@
   </si>
   <si>
     <t>755-KTR10EZPF6042</t>
+  </si>
+  <si>
+    <t>Distanzbolzen</t>
+  </si>
+  <si>
+    <t>B 080805 PC-V0-G 7035</t>
+  </si>
+  <si>
+    <t>DIBLZ AK 30x5/IM3/10</t>
+  </si>
+  <si>
+    <t>59006986</t>
+  </si>
+  <si>
+    <t>Schraube M3x6</t>
+  </si>
+  <si>
+    <t>SHR-ZYL-ISO14580-A2/70-TX10-M3X6</t>
+  </si>
+  <si>
+    <t>52041060</t>
+  </si>
+  <si>
+    <t>96021115</t>
   </si>
 </sst>
 </file>
@@ -2449,7 +2440,7 @@
     </row>
     <row r="2" spans="1:9" s="23" customFormat="1" ht="19.899999999999999" customHeight="1">
       <c r="A2" s="103" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B2" s="103"/>
       <c r="C2" s="103"/>
@@ -2459,7 +2450,7 @@
       <c r="G2" s="103"/>
       <c r="H2" s="101">
         <f ca="1">TODAY()</f>
-        <v>44030</v>
+        <v>44035</v>
       </c>
       <c r="I2" s="101"/>
     </row>
@@ -2472,7 +2463,7 @@
       <c r="F3" s="60"/>
       <c r="G3" s="38"/>
       <c r="H3" s="102" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="I3" s="102"/>
     </row>
@@ -2507,28 +2498,28 @@
     </row>
     <row r="5" spans="1:9" s="15" customFormat="1">
       <c r="A5" s="81" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="B5" s="64" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="65" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="64" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="65" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="65" t="s">
+      <c r="G5" s="65" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="64" t="s">
+      <c r="H5" s="67" t="s">
         <v>79</v>
-      </c>
-      <c r="E5" s="65" t="s">
-        <v>80</v>
-      </c>
-      <c r="F5" s="65" t="s">
-        <v>81</v>
-      </c>
-      <c r="G5" s="65" t="s">
-        <v>82</v>
-      </c>
-      <c r="H5" s="67" t="s">
-        <v>83</v>
       </c>
       <c r="I5" s="67">
         <v>1</v>
@@ -2536,28 +2527,28 @@
     </row>
     <row r="6" spans="1:9" s="15" customFormat="1">
       <c r="A6" s="81" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B6" s="63" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C6" s="68" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D6" s="73" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E6" s="68" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F6" s="68" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G6" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" s="70" t="s">
         <v>82</v>
-      </c>
-      <c r="H6" s="70" t="s">
-        <v>86</v>
       </c>
       <c r="I6" s="70">
         <v>4</v>
@@ -2565,28 +2556,28 @@
     </row>
     <row r="7" spans="1:9" s="15" customFormat="1">
       <c r="A7" s="81" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B7" s="63" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C7" s="71" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E7" s="68" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F7" s="68" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G7" s="68" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H7" s="72" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I7" s="70">
         <v>2</v>
@@ -2594,28 +2585,28 @@
     </row>
     <row r="8" spans="1:9" s="15" customFormat="1" ht="25.5">
       <c r="A8" s="81" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B8" s="63" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" s="71" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="73" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="68" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="68" t="s">
         <v>91</v>
       </c>
-      <c r="C8" s="71" t="s">
+      <c r="G8" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H8" s="70" t="s">
         <v>92</v>
-      </c>
-      <c r="D8" s="73" t="s">
-        <v>93</v>
-      </c>
-      <c r="E8" s="68" t="s">
-        <v>94</v>
-      </c>
-      <c r="F8" s="68" t="s">
-        <v>95</v>
-      </c>
-      <c r="G8" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H8" s="70" t="s">
-        <v>96</v>
       </c>
       <c r="I8" s="70">
         <v>1</v>
@@ -2623,28 +2614,28 @@
     </row>
     <row r="9" spans="1:9" s="15" customFormat="1">
       <c r="A9" s="81" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B9" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" s="71" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" s="73" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" s="68" t="s">
+        <v>96</v>
+      </c>
+      <c r="F9" s="68" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="71" t="s">
+      <c r="G9" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" s="70" t="s">
         <v>98</v>
-      </c>
-      <c r="D9" s="73" t="s">
-        <v>99</v>
-      </c>
-      <c r="E9" s="68" t="s">
-        <v>100</v>
-      </c>
-      <c r="F9" s="68" t="s">
-        <v>101</v>
-      </c>
-      <c r="G9" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H9" s="70" t="s">
-        <v>102</v>
       </c>
       <c r="I9" s="70">
         <v>2</v>
@@ -2652,28 +2643,28 @@
     </row>
     <row r="10" spans="1:9" s="15" customFormat="1">
       <c r="A10" s="81" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B10" s="63" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="C10" s="71" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="D10" s="73" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="E10" s="68" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="F10" s="68" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="G10" s="68" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H10" s="70" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="I10" s="70">
         <v>1</v>
@@ -2681,28 +2672,28 @@
     </row>
     <row r="11" spans="1:9" s="15" customFormat="1">
       <c r="A11" s="81" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B11" s="63" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="C11" s="68" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="73" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="68" t="s">
+        <v>101</v>
+      </c>
+      <c r="F11" s="68" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="72" t="s">
         <v>103</v>
-      </c>
-      <c r="D11" s="73" t="s">
-        <v>104</v>
-      </c>
-      <c r="E11" s="68" t="s">
-        <v>105</v>
-      </c>
-      <c r="F11" s="68" t="s">
-        <v>106</v>
-      </c>
-      <c r="G11" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H11" s="72" t="s">
-        <v>107</v>
       </c>
       <c r="I11" s="70">
         <v>1</v>
@@ -2710,28 +2701,28 @@
     </row>
     <row r="12" spans="1:9" s="15" customFormat="1" ht="38.25">
       <c r="A12" s="63" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B12" s="63" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="C12" s="68" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="73" t="s">
+        <v>105</v>
+      </c>
+      <c r="E12" s="68" t="s">
+        <v>106</v>
+      </c>
+      <c r="F12" s="68" t="s">
+        <v>107</v>
+      </c>
+      <c r="G12" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H12" s="72" t="s">
         <v>108</v>
-      </c>
-      <c r="D12" s="73" t="s">
-        <v>109</v>
-      </c>
-      <c r="E12" s="68" t="s">
-        <v>110</v>
-      </c>
-      <c r="F12" s="68" t="s">
-        <v>111</v>
-      </c>
-      <c r="G12" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H12" s="72" t="s">
-        <v>112</v>
       </c>
       <c r="I12" s="70">
         <v>1</v>
@@ -2739,28 +2730,28 @@
     </row>
     <row r="13" spans="1:9" s="15" customFormat="1">
       <c r="A13" s="81" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B13" s="63" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="C13" s="68" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D13" s="73" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="E13" s="68" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F13" s="68" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G13" s="68" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I13" s="70">
         <v>1</v>
@@ -2768,28 +2759,28 @@
     </row>
     <row r="14" spans="1:9" s="15" customFormat="1">
       <c r="A14" s="81" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B14" s="63" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="C14" s="73" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14" s="73" t="s">
+        <v>114</v>
+      </c>
+      <c r="E14" s="68" t="s">
+        <v>115</v>
+      </c>
+      <c r="F14" s="68" t="s">
+        <v>116</v>
+      </c>
+      <c r="G14" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H14" s="70" t="s">
         <v>117</v>
-      </c>
-      <c r="D14" s="73" t="s">
-        <v>118</v>
-      </c>
-      <c r="E14" s="68" t="s">
-        <v>119</v>
-      </c>
-      <c r="F14" s="68" t="s">
-        <v>120</v>
-      </c>
-      <c r="G14" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" s="70" t="s">
-        <v>121</v>
       </c>
       <c r="I14" s="70">
         <v>1</v>
@@ -2797,28 +2788,28 @@
     </row>
     <row r="15" spans="1:9" s="15" customFormat="1">
       <c r="A15" s="81" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B15" s="63" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C15" s="71" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="D15" s="63" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E15" s="71" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F15" s="71" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="G15" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="I15" s="70">
         <v>1</v>
@@ -2826,26 +2817,26 @@
     </row>
     <row r="16" spans="1:9" s="15" customFormat="1">
       <c r="A16" s="84" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B16" s="85"/>
       <c r="C16" s="86" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D16" s="85" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F16" s="86" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G16" s="86" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H16" s="87" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I16" s="87">
         <v>1</v>
@@ -2853,28 +2844,28 @@
     </row>
     <row r="17" spans="1:9" s="15" customFormat="1" ht="15" customHeight="1">
       <c r="A17" s="81" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B17" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="71" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="E17" s="71" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="71" t="s">
+        <v>128</v>
+      </c>
+      <c r="G17" s="71" t="s">
+        <v>78</v>
+      </c>
+      <c r="H17" s="70" t="s">
         <v>129</v>
-      </c>
-      <c r="C17" s="71" t="s">
-        <v>130</v>
-      </c>
-      <c r="D17" s="63" t="s">
-        <v>131</v>
-      </c>
-      <c r="E17" s="71" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="G17" s="71" t="s">
-        <v>82</v>
-      </c>
-      <c r="H17" s="70" t="s">
-        <v>133</v>
       </c>
       <c r="I17" s="70">
         <v>2</v>
@@ -2882,28 +2873,28 @@
     </row>
     <row r="18" spans="1:9" s="15" customFormat="1">
       <c r="A18" s="96" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B18" s="97" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C18" s="97" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D18" s="97" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E18" s="98" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F18" s="97" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="G18" s="98" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H18" s="99" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="I18" s="100">
         <v>1</v>
@@ -2911,28 +2902,28 @@
     </row>
     <row r="19" spans="1:9" s="15" customFormat="1" ht="15" customHeight="1">
       <c r="A19" s="81" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="B19" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C19" s="63" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="D19" s="63" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E19" s="71" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F19" s="63" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="G19" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H19" s="72" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="I19" s="70">
         <v>1</v>
@@ -2940,28 +2931,28 @@
     </row>
     <row r="20" spans="1:9" s="15" customFormat="1">
       <c r="A20" s="81" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B20" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C20" s="63" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="D20" s="63" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E20" s="71" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F20" s="63" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="G20" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H20" s="72" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="I20" s="70">
         <v>1</v>
@@ -2969,28 +2960,28 @@
     </row>
     <row r="21" spans="1:9" s="15" customFormat="1">
       <c r="A21" s="81" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B21" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C21" s="63" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="D21" s="63" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E21" s="71" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="F21" s="63" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="G21" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H21" s="72" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="I21" s="70">
         <v>1</v>
@@ -2998,28 +2989,28 @@
     </row>
     <row r="22" spans="1:9" s="15" customFormat="1">
       <c r="A22" s="81" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B22" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C22" s="63" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="D22" s="63" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E22" s="63" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F22" s="63" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G22" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H22" s="72" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="I22" s="70">
         <v>1</v>
@@ -3027,28 +3018,28 @@
     </row>
     <row r="23" spans="1:9" s="15" customFormat="1">
       <c r="A23" s="81" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="B23" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C23" s="63" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="D23" s="63" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E23" s="63" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F23" s="63" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="G23" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H23" s="72" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="I23" s="70">
         <v>1</v>
@@ -3056,28 +3047,28 @@
     </row>
     <row r="24" spans="1:9" s="15" customFormat="1">
       <c r="A24" s="81" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B24" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C24" s="63" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="D24" s="63" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E24" s="71" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F24" s="63" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="G24" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H24" s="72" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="I24" s="70">
         <v>1</v>
@@ -3085,28 +3076,28 @@
     </row>
     <row r="25" spans="1:9" s="15" customFormat="1" ht="25.5">
       <c r="A25" s="81" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="B25" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C25" s="63" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D25" s="63" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E25" s="71" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F25" s="63" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="G25" s="71" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H25" s="72" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="I25" s="70">
         <v>6</v>
@@ -3114,28 +3105,28 @@
     </row>
     <row r="26" spans="1:9" s="15" customFormat="1">
       <c r="A26" s="81" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B26" s="63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C26" s="68" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="D26" s="73" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E26" s="68" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F26" s="68" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="G26" s="68" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H26" s="75" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="I26" s="70">
         <v>1</v>
@@ -3143,28 +3134,28 @@
     </row>
     <row r="27" spans="1:9" s="15" customFormat="1">
       <c r="A27" s="81" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B27" s="63" t="s">
+        <v>140</v>
+      </c>
+      <c r="C27" s="68" t="s">
+        <v>126</v>
+      </c>
+      <c r="D27" s="73" t="s">
+        <v>141</v>
+      </c>
+      <c r="E27" s="68" t="s">
+        <v>142</v>
+      </c>
+      <c r="F27" s="68" t="s">
+        <v>143</v>
+      </c>
+      <c r="G27" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H27" s="75" t="s">
         <v>144</v>
-      </c>
-      <c r="C27" s="68" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="73" t="s">
-        <v>145</v>
-      </c>
-      <c r="E27" s="68" t="s">
-        <v>146</v>
-      </c>
-      <c r="F27" s="68" t="s">
-        <v>147</v>
-      </c>
-      <c r="G27" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H27" s="75" t="s">
-        <v>148</v>
       </c>
       <c r="I27" s="70">
         <v>1</v>
@@ -3172,28 +3163,28 @@
     </row>
     <row r="28" spans="1:9" s="15" customFormat="1" ht="25.5">
       <c r="A28" s="81" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B28" s="63" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="C28" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="D28" s="73" t="s">
+        <v>146</v>
+      </c>
+      <c r="E28" s="68" t="s">
+        <v>147</v>
+      </c>
+      <c r="F28" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="G28" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="H28" s="75" t="s">
         <v>149</v>
-      </c>
-      <c r="D28" s="73" t="s">
-        <v>150</v>
-      </c>
-      <c r="E28" s="68" t="s">
-        <v>151</v>
-      </c>
-      <c r="F28" s="68" t="s">
-        <v>152</v>
-      </c>
-      <c r="G28" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H28" s="75" t="s">
-        <v>153</v>
       </c>
       <c r="I28" s="70">
         <v>1</v>
@@ -3201,26 +3192,26 @@
     </row>
     <row r="29" spans="1:9" s="15" customFormat="1">
       <c r="A29" s="84" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B29" s="85"/>
       <c r="C29" s="86" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D29" s="85" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E29" s="86" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F29" s="86" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="G29" s="86" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H29" s="87" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="I29" s="87">
         <v>1</v>
@@ -3228,26 +3219,26 @@
     </row>
     <row r="30" spans="1:9" s="15" customFormat="1">
       <c r="A30" s="84" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B30" s="85"/>
       <c r="C30" s="86" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D30" s="85" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E30" s="86" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F30" s="86" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G30" s="86" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H30" s="87" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I30" s="87">
         <v>1</v>
@@ -3304,10 +3295,10 @@
     </row>
     <row r="35" spans="1:9" s="15" customFormat="1">
       <c r="A35" s="82" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B35" s="83" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="5"/>
@@ -3469,7 +3460,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="48.6" customHeight="1">
       <c r="A1" s="104" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B1" s="104"/>
       <c r="C1" s="58"/>
@@ -3488,7 +3479,7 @@
       <c r="E2" s="103"/>
       <c r="F2" s="79">
         <f ca="1">TODAY()</f>
-        <v>44030</v>
+        <v>44035</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="23" customFormat="1" ht="19.899999999999999" customHeight="1">
@@ -3530,13 +3521,13 @@
         <v>44</v>
       </c>
       <c r="C5" s="77" t="s">
-        <v>45</v>
+        <v>296</v>
       </c>
       <c r="D5" s="66" t="s">
         <v>44</v>
       </c>
       <c r="E5" s="66" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="F5" s="70">
         <v>1</v>
@@ -3544,19 +3535,19 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="80" t="s">
-        <v>46</v>
+        <v>295</v>
       </c>
       <c r="B6" s="68" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C6" s="77" t="s">
-        <v>48</v>
+        <v>297</v>
       </c>
       <c r="D6" s="69" t="s">
-        <v>82</v>
-      </c>
-      <c r="E6" s="69" t="s">
-        <v>240</v>
+        <v>44</v>
+      </c>
+      <c r="E6" s="77" t="s">
+        <v>298</v>
       </c>
       <c r="F6" s="70">
         <v>2</v>
@@ -3564,19 +3555,19 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="80" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B7" s="68" t="s">
         <v>44</v>
       </c>
       <c r="C7" s="89" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D7" s="69" t="s">
         <v>44</v>
       </c>
       <c r="E7" s="69" t="s">
-        <v>50</v>
+        <v>301</v>
       </c>
       <c r="F7" s="70">
         <v>1</v>
@@ -3584,19 +3575,19 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="80" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B8" s="63" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C8" s="74" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D8" s="69" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E8" s="69" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F8" s="75">
         <v>1</v>
@@ -3604,19 +3595,19 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="71" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B9" s="63" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C9" s="74" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D9" s="69" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E9" s="69" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F9" s="75">
         <v>1</v>
@@ -3624,19 +3615,19 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="71" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="B10" s="63" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="C10" s="74" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D10" s="69" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="E10" s="69" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="F10" s="75">
         <v>1</v>
@@ -3644,39 +3635,27 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="63" t="s">
-        <v>163</v>
+        <v>299</v>
       </c>
       <c r="B11" s="63"/>
       <c r="C11" s="69"/>
       <c r="D11" s="69" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="E11" s="69" t="s">
-        <v>238</v>
+        <v>300</v>
       </c>
       <c r="F11" s="75">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="63" t="s">
-        <v>164</v>
-      </c>
-      <c r="B12" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" s="69" t="s">
-        <v>165</v>
-      </c>
-      <c r="D12" s="69" t="s">
-        <v>166</v>
-      </c>
-      <c r="E12" s="69" t="s">
-        <v>167</v>
-      </c>
-      <c r="F12" s="75">
-        <v>1</v>
-      </c>
+      <c r="A12" s="63"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="69"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="75"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="63"/>
@@ -3969,7 +3948,7 @@
       <c r="C2" s="38"/>
       <c r="D2" s="33">
         <f ca="1">Stückliste!H2</f>
-        <v>44030</v>
+        <v>44035</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="22" customFormat="1" ht="19.899999999999999" customHeight="1">
@@ -3996,7 +3975,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C5" s="26"/>
       <c r="D5" s="27"/>
@@ -4076,7 +4055,7 @@
         <v>28</v>
       </c>
       <c r="B13" s="44" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C13" s="26"/>
       <c r="D13" s="27"/>
@@ -6121,7 +6100,7 @@
       <c r="D2" s="103"/>
       <c r="E2" s="33">
         <f ca="1">Stückliste!H2</f>
-        <v>44030</v>
+        <v>44035</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="6" customFormat="1" ht="19.899999999999999" customHeight="1">
@@ -6153,580 +6132,580 @@
     </row>
     <row r="5" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A5" s="63" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="B5" s="63" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="C5" s="68" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D5" s="69" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E5" s="68" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A6" s="63" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B6" s="63" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="C6" s="68" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D6" s="69" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E6" s="68" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A7" s="63" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="B7" s="63" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="C7" s="68" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="D7" s="69" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E7" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A8" s="63" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="B8" s="63" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="C8" s="68" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="D8" s="69" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E8" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A9" s="63" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="B9" s="63" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="C9" s="68" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="D9" s="69" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E9" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A10" s="63" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B10" s="63" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="C10" s="68" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="D10" s="69" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E10" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A11" s="63" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="B11" s="63" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="D11" s="69" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E11" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A12" s="63" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="B12" s="63" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C12" s="68" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="D12" s="69" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E12" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A13" s="63" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="B13" s="63" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="C13" s="68" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="D13" s="69" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E13" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A14" s="63" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="B14" s="63" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="C14" s="68" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="D14" s="69" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E14" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A15" s="63" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B15" s="63" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="C15" s="68" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="D15" s="69" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E15" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A16" s="63" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="B16" s="63" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="C16" s="68" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="D16" s="69" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E16" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A17" s="63" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B17" s="63" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="C17" s="68" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="D17" s="69" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E17" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A18" s="63" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B18" s="63" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="C18" s="68" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D18" s="69" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E18" s="68" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A19" s="39" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B19" s="93" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="C19" s="94" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="D19" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E19" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A20" s="39" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B20" s="93" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="C20" s="94" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="D20" s="94" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="22" customFormat="1" ht="15" customHeight="1">
       <c r="A21" s="39" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B21" s="93" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="C21" s="95" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="D21" s="95" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15" customHeight="1">
       <c r="A22" s="39" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B22" s="93" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="C22" s="94" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="D22" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15" customHeight="1">
       <c r="A23" s="39" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="B23" s="93" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="C23" s="94" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="D23" s="94" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15" customHeight="1">
       <c r="A24" s="39" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="B24" s="93" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="C24" s="95" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="D24" s="95" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15" customHeight="1">
       <c r="A25" s="39" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B25" s="93" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="C25" s="94" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="D25" s="94" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15" customHeight="1">
       <c r="A26" s="39" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B26" s="93" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="C26" s="94" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="D26" s="94" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E26" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15" customHeight="1">
       <c r="A27" s="39" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B27" s="93" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="C27" s="95" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="D27" s="95" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="15" customHeight="1">
       <c r="A28" s="39" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B28" s="93" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C28" s="94" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E28" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15" customHeight="1">
       <c r="A29" s="39" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="B29" s="93" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="C29" s="94" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="D29" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" customHeight="1">
       <c r="A30" s="39" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="B30" s="93" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C30" s="95" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="D30" s="95" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E30" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15" customHeight="1">
       <c r="A31" s="39" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="B31" s="93" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C31" s="94" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="D31" s="94" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15" customHeight="1">
       <c r="A32" s="39" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="B32" s="93" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C32" s="94" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="D32" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E32" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" customHeight="1">
       <c r="A33" s="39" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B33" s="93" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="C33" s="95" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D33" s="95" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" customHeight="1">
       <c r="A34" s="39" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B34" s="93" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="C34" s="94" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="D34" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E34" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" customHeight="1">
       <c r="A35" s="39" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="B35" s="93" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="C35" s="94" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="D35" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E35" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15" customHeight="1">
       <c r="A36" s="39" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="B36" s="93" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="C36" s="95" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="D36" s="95" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E36" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15" customHeight="1">
       <c r="A37" s="39" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B37" s="93" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="C37" s="94" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="D37" s="94" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E37" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" customHeight="1">
       <c r="A38" s="39" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B38" s="93" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="C38" s="94" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="D38" s="94" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E38" s="39" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" customHeight="1">

</xml_diff>